<commit_message>
feat: estructura inicial del proyecto con componentes React
</commit_message>
<xml_diff>
--- a/UBICACION_HAMBURGUESAS.xlsx
+++ b/UBICACION_HAMBURGUESAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zelda\Documents\ESTUDIO PROGRAMACION\CREAR PAGINA DE RUTA DE HAMBURGUESAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E7C5459-F916-40FF-B9C0-2EC1F897E977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{336994BD-6B38-406C-92A9-4D09747578B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8FA2386E-D48D-451C-B4F4-F556A3A8FF81}"/>
+    <workbookView xWindow="12570" yWindow="585" windowWidth="16230" windowHeight="14190" xr2:uid="{8FA2386E-D48D-451C-B4F4-F556A3A8FF81}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -254,9 +254,6 @@
     <t>Sitio websitio web</t>
   </si>
   <si>
-    <t>Teléfonoteléfono</t>
-  </si>
-  <si>
     <t>ROCK BURGUER</t>
   </si>
   <si>
@@ -402,6 +399,9 @@
   </si>
   <si>
     <t>Ciudad</t>
+  </si>
+  <si>
+    <t>Teléfono</t>
   </si>
 </sst>
 </file>
@@ -509,7 +509,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -522,9 +522,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -895,28 +892,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -925,10 +922,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
@@ -999,21 +996,21 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1119,7 +1116,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>40</v>
@@ -1146,7 +1143,7 @@
         <v>43</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>14</v>
@@ -1215,10 +1212,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>14</v>
@@ -1289,7 +1286,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>62</v>
@@ -1328,26 +1325,26 @@
         <v>68</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="2">
         <v>3162948685</v>
       </c>
@@ -1355,23 +1352,23 @@
         <v>27</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="10"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="2">
         <v>3175738174</v>
       </c>
@@ -1379,7 +1376,7 @@
         <v>27</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="33" x14ac:dyDescent="0.25">
@@ -1387,23 +1384,23 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="10"/>
-      <c r="F21" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="G21" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
@@ -1411,141 +1408,141 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="10"/>
-      <c r="F22" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="G22" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="9"/>
+      <c r="F23" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="10"/>
-      <c r="F23" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="G23" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H23" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="H23" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="9"/>
+      <c r="F24" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="G24" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H24" s="7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="H24" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="9"/>
+      <c r="F25" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="10"/>
-      <c r="F25" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="G25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H25" s="6"/>
+      <c r="H25" s="5"/>
     </row>
     <row r="26" spans="1:8" ht="33" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="9"/>
+      <c r="F26" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E26" s="10"/>
-      <c r="F26" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="G26" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="9"/>
+      <c r="F27" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="G27" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="33" x14ac:dyDescent="0.25">
@@ -1555,23 +1552,23 @@
       <c r="B28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="11" t="s">
         <v>13</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>